<commit_message>
Update examples per B18
</commit_message>
<xml_diff>
--- a/examples/schedule_prep_spreadsheet.xlsx
+++ b/examples/schedule_prep_spreadsheet.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jpadams/proj/pds/pdsen/workspace/lasso-issues/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{923B8CAF-0916-CC42-959C-D375AB02026B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14DE344-07C9-9940-92E8-B762D77CA847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="940" windowWidth="33240" windowHeight="15540" activeTab="1" xr2:uid="{77BE7B00-5D39-0F40-9AE5-E33691EB16DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Release Date" sheetId="3" r:id="rId1"/>
-    <sheet name="b17_schedule_prep_spreadsheet" sheetId="2" r:id="rId2"/>
-    <sheet name="Baseline" sheetId="1" r:id="rId3"/>
+    <sheet name="b18_schedule_prep_spreadsheet" sheetId="4" r:id="rId2"/>
+    <sheet name="b17_schedule_prep_spreadsheet" sheetId="2" r:id="rId3"/>
+    <sheet name="Baseline" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Baseline!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Baseline!$A$1:$H$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="88">
   <si>
     <t xml:space="preserve">Task </t>
   </si>
@@ -701,7 +702,7 @@
         <v>33</v>
       </c>
       <c r="B1" s="4">
-        <v>46177</v>
+        <v>46366</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -713,6 +714,766 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96C7D9C4-D69C-794B-81EF-3216314ED497}">
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="55.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="18.5" customWidth="1"/>
+    <col min="9" max="9" width="83.1640625" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="4">
+        <f t="shared" ref="C2:C19" si="0">D2-E2</f>
+        <v>46094</v>
+      </c>
+      <c r="D2" s="4">
+        <f>'Release Date'!$B$1-F2</f>
+        <v>46135</v>
+      </c>
+      <c r="E2" s="3">
+        <v>41</v>
+      </c>
+      <c r="F2">
+        <v>231</v>
+      </c>
+      <c r="G2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="2" t="b">
+        <f>IF(C2="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C2+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="b">
+        <f>IF(D2="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D2),21)=0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D3" s="4">
+        <f>'Release Date'!$B$1-F3</f>
+        <v>46282</v>
+      </c>
+      <c r="E3" s="3">
+        <v>167</v>
+      </c>
+      <c r="F3">
+        <v>84</v>
+      </c>
+      <c r="G3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D4" s="4">
+        <f>'Release Date'!$B$1-F4</f>
+        <v>46282</v>
+      </c>
+      <c r="E4" s="3">
+        <v>167</v>
+      </c>
+      <c r="F4">
+        <v>84</v>
+      </c>
+      <c r="G4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="2" t="b">
+        <f>IF(C4="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C4+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="b">
+        <f>IF(D4="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D4),21)=0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D5" s="4">
+        <f>'Release Date'!$B$1-F5</f>
+        <v>46282</v>
+      </c>
+      <c r="E5" s="3">
+        <v>167</v>
+      </c>
+      <c r="F5">
+        <v>84</v>
+      </c>
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" s="2" t="b">
+        <f>IF(C5="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C5+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="b">
+        <f>IF(D5="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D5),21)=0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D6" s="4">
+        <f>'Release Date'!$B$1-F6</f>
+        <v>46282</v>
+      </c>
+      <c r="E6" s="3">
+        <v>167</v>
+      </c>
+      <c r="F6">
+        <v>84</v>
+      </c>
+      <c r="G6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="2" t="b">
+        <f>IF(C6="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C6+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="b">
+        <f>IF(D6="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D6),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D7" s="4">
+        <f>'Release Date'!$B$1-F7</f>
+        <v>46282</v>
+      </c>
+      <c r="E7" s="3">
+        <v>167</v>
+      </c>
+      <c r="F7">
+        <v>84</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" s="2" t="b">
+        <f>IF(C7="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C7+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="b">
+        <f>IF(D7="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D7),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4">
+        <f t="shared" si="0"/>
+        <v>46115</v>
+      </c>
+      <c r="D8" s="4">
+        <f>'Release Date'!$B$1-F8</f>
+        <v>46303</v>
+      </c>
+      <c r="E8">
+        <v>188</v>
+      </c>
+      <c r="F8">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="2" t="b">
+        <f>IF(C8="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C8+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="b">
+        <f>IF(D8="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D8),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="4">
+        <f t="shared" si="0"/>
+        <v>46282</v>
+      </c>
+      <c r="D9" s="4">
+        <f>'Release Date'!$B$1-F9</f>
+        <v>46282</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>84</v>
+      </c>
+      <c r="G9" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="2" t="b">
+        <f>IF(C9="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C9+20)),21)=0))</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="b">
+        <f>IF(D9="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D9),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="4">
+        <f t="shared" si="0"/>
+        <v>46283</v>
+      </c>
+      <c r="D10" s="4">
+        <f>'Release Date'!$B$1-F10</f>
+        <v>46303</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>63</v>
+      </c>
+      <c r="G10" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" s="2" t="b">
+        <f>IF(C10="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C10+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="b">
+        <f>IF(D10="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D10),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="4">
+        <f t="shared" si="0"/>
+        <v>46283</v>
+      </c>
+      <c r="D11" s="4">
+        <f>'Release Date'!$B$1-F11</f>
+        <v>46303</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="shared" si="0"/>
+        <v>46283</v>
+      </c>
+      <c r="D12" s="4">
+        <f>'Release Date'!$B$1-F12</f>
+        <v>46303</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>63</v>
+      </c>
+      <c r="G12" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" t="s">
+        <v>60</v>
+      </c>
+      <c r="J12" s="2" t="b">
+        <f>IF(C12="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C12+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="b">
+        <f>IF(D12="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D12),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="4">
+        <f t="shared" si="0"/>
+        <v>46283</v>
+      </c>
+      <c r="D13" s="4">
+        <f>'Release Date'!$B$1-F13</f>
+        <v>46303</v>
+      </c>
+      <c r="E13">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>63</v>
+      </c>
+      <c r="G13" t="s">
+        <v>36</v>
+      </c>
+      <c r="H13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" t="s">
+        <v>60</v>
+      </c>
+      <c r="J13" s="2" t="b">
+        <f>IF(C13="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C13+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="b">
+        <f>IF(D13="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D13),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4">
+        <f t="shared" si="0"/>
+        <v>46304</v>
+      </c>
+      <c r="D14" s="4">
+        <f>'Release Date'!$B$1-F14</f>
+        <v>46345</v>
+      </c>
+      <c r="E14">
+        <v>41</v>
+      </c>
+      <c r="F14">
+        <v>21</v>
+      </c>
+      <c r="G14" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="2" t="b">
+        <f>IF(C14="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C14+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="b">
+        <f>IF(D14="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D14),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="4">
+        <f t="shared" si="0"/>
+        <v>46304</v>
+      </c>
+      <c r="D15" s="4">
+        <f>'Release Date'!$B$1-F15</f>
+        <v>46345</v>
+      </c>
+      <c r="E15">
+        <v>41</v>
+      </c>
+      <c r="F15">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" s="2" t="b">
+        <f>IF(C15="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C15+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="b">
+        <f>IF(D15="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D15),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="4">
+        <f t="shared" si="0"/>
+        <v>46304</v>
+      </c>
+      <c r="D16" s="4">
+        <f>'Release Date'!$B$1-F16</f>
+        <v>46345</v>
+      </c>
+      <c r="E16">
+        <v>41</v>
+      </c>
+      <c r="F16">
+        <v>21</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" t="s">
+        <v>61</v>
+      </c>
+      <c r="J16" s="2" t="b">
+        <f>IF(C16="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C16+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="b">
+        <f>IF(D16="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D16),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="4">
+        <f t="shared" si="0"/>
+        <v>46304</v>
+      </c>
+      <c r="D17" s="4">
+        <f>'Release Date'!$B$1-F17</f>
+        <v>46325</v>
+      </c>
+      <c r="E17">
+        <v>21</v>
+      </c>
+      <c r="F17">
+        <v>41</v>
+      </c>
+      <c r="G17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" s="2" t="b">
+        <f>IF(C17="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C17+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="b">
+        <f>IF(D17="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D17),21)=0))</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="4">
+        <f t="shared" si="0"/>
+        <v>46325</v>
+      </c>
+      <c r="D18" s="4">
+        <f>'Release Date'!$B$1-F18</f>
+        <v>46366</v>
+      </c>
+      <c r="E18">
+        <v>41</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J18" s="2" t="b">
+        <f>IF(C18="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C18+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="b">
+        <f>IF(D18="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D18),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="4">
+        <f t="shared" si="0"/>
+        <v>46346</v>
+      </c>
+      <c r="D19" s="4">
+        <f>'Release Date'!$B$1-F19</f>
+        <v>46366</v>
+      </c>
+      <c r="E19">
+        <v>20</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" t="s">
+        <v>61</v>
+      </c>
+      <c r="J19" s="2" t="b">
+        <f>IF(C19="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,(C19+20)),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="b">
+        <f>IF(D19="","",(MOD(_xlfn.DAYS('Release Date'!$B$1,D19),21)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7A282D7-36CC-A540-8420-FCD049761715}">
   <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -770,11 +1531,11 @@
       </c>
       <c r="C2" s="4">
         <f t="shared" ref="C2:C3" si="0">D2-E2</f>
-        <v>45905</v>
+        <v>46094</v>
       </c>
       <c r="D2" s="4">
         <f>'Release Date'!$B$1-F2</f>
-        <v>45946</v>
+        <v>46135</v>
       </c>
       <c r="E2" s="3">
         <v>41</v>
@@ -806,11 +1567,11 @@
       </c>
       <c r="C3" s="4">
         <f t="shared" si="0"/>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D3" s="4">
         <f>'Release Date'!$B$1-F3</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E3" s="3">
         <v>167</v>
@@ -836,11 +1597,11 @@
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4" si="1">D4-E4</f>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D4" s="4">
         <f>'Release Date'!$B$1-F4</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E4" s="3">
         <v>167</v>
@@ -872,11 +1633,11 @@
       </c>
       <c r="C5" s="4">
         <f t="shared" ref="C5:C6" si="2">D5-E5</f>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D5" s="4">
         <f>'Release Date'!$B$1-F5</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E5" s="3">
         <v>167</v>
@@ -908,11 +1669,11 @@
       </c>
       <c r="C6" s="4">
         <f t="shared" si="2"/>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D6" s="4">
         <f>'Release Date'!$B$1-F6</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E6" s="3">
         <v>167</v>
@@ -945,11 +1706,11 @@
       </c>
       <c r="C7" s="4">
         <f t="shared" ref="C7:C19" si="3">D7-E7</f>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D7" s="4">
         <f>'Release Date'!$B$1-F7</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E7" s="3">
         <v>167</v>
@@ -982,11 +1743,11 @@
       </c>
       <c r="C8" s="4">
         <f t="shared" si="3"/>
-        <v>45926</v>
+        <v>46115</v>
       </c>
       <c r="D8" s="4">
         <f>'Release Date'!$B$1-F8</f>
-        <v>46114</v>
+        <v>46303</v>
       </c>
       <c r="E8">
         <v>188</v>
@@ -1019,11 +1780,11 @@
       </c>
       <c r="C9" s="4">
         <f t="shared" si="3"/>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="D9" s="4">
         <f>'Release Date'!$B$1-F9</f>
-        <v>46093</v>
+        <v>46282</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1056,11 +1817,11 @@
       </c>
       <c r="C10" s="4">
         <f t="shared" ref="C10:C11" si="4">D10-E10</f>
-        <v>46094</v>
+        <v>46283</v>
       </c>
       <c r="D10" s="4">
         <f>'Release Date'!$B$1-F10</f>
-        <v>46114</v>
+        <v>46303</v>
       </c>
       <c r="E10">
         <v>20</v>
@@ -1096,11 +1857,11 @@
       </c>
       <c r="C11" s="4">
         <f t="shared" si="4"/>
-        <v>46094</v>
+        <v>46283</v>
       </c>
       <c r="D11" s="4">
         <f>'Release Date'!$B$1-F11</f>
-        <v>46114</v>
+        <v>46303</v>
       </c>
       <c r="E11">
         <v>20</v>
@@ -1127,11 +1888,11 @@
       </c>
       <c r="C12" s="4">
         <f t="shared" si="3"/>
-        <v>46094</v>
+        <v>46283</v>
       </c>
       <c r="D12" s="4">
         <f>'Release Date'!$B$1-F12</f>
-        <v>46114</v>
+        <v>46303</v>
       </c>
       <c r="E12">
         <v>20</v>
@@ -1167,11 +1928,11 @@
       </c>
       <c r="C13" s="4">
         <f t="shared" si="3"/>
-        <v>46094</v>
+        <v>46283</v>
       </c>
       <c r="D13" s="4">
         <f>'Release Date'!$B$1-F13</f>
-        <v>46114</v>
+        <v>46303</v>
       </c>
       <c r="E13">
         <v>20</v>
@@ -1207,11 +1968,11 @@
       </c>
       <c r="C14" s="4">
         <f t="shared" si="3"/>
-        <v>46115</v>
+        <v>46304</v>
       </c>
       <c r="D14" s="4">
         <f>'Release Date'!$B$1-F14</f>
-        <v>46156</v>
+        <v>46345</v>
       </c>
       <c r="E14">
         <v>41</v>
@@ -1247,11 +2008,11 @@
       </c>
       <c r="C15" s="4">
         <f t="shared" si="3"/>
-        <v>46115</v>
+        <v>46304</v>
       </c>
       <c r="D15" s="4">
         <f>'Release Date'!$B$1-F15</f>
-        <v>46156</v>
+        <v>46345</v>
       </c>
       <c r="E15">
         <v>41</v>
@@ -1287,11 +2048,11 @@
       </c>
       <c r="C16" s="4">
         <f t="shared" si="3"/>
-        <v>46115</v>
+        <v>46304</v>
       </c>
       <c r="D16" s="4">
         <f>'Release Date'!$B$1-F16</f>
-        <v>46156</v>
+        <v>46345</v>
       </c>
       <c r="E16">
         <v>41</v>
@@ -1327,11 +2088,11 @@
       </c>
       <c r="C17" s="4">
         <f t="shared" si="3"/>
-        <v>46115</v>
+        <v>46304</v>
       </c>
       <c r="D17" s="4">
         <f>'Release Date'!$B$1-F17</f>
-        <v>46136</v>
+        <v>46325</v>
       </c>
       <c r="E17">
         <v>21</v>
@@ -1364,11 +2125,11 @@
       </c>
       <c r="C18" s="4">
         <f t="shared" si="3"/>
-        <v>46136</v>
+        <v>46325</v>
       </c>
       <c r="D18" s="4">
         <f>'Release Date'!$B$1-F18</f>
-        <v>46177</v>
+        <v>46366</v>
       </c>
       <c r="E18">
         <v>41</v>
@@ -1404,11 +2165,11 @@
       </c>
       <c r="C19" s="4">
         <f t="shared" si="3"/>
-        <v>46157</v>
+        <v>46346</v>
       </c>
       <c r="D19" s="4">
         <f>'Release Date'!$B$1-F19</f>
-        <v>46177</v>
+        <v>46366</v>
       </c>
       <c r="E19">
         <v>20</v>
@@ -1472,7 +2233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1773B976-BCDA-D945-919B-7C561A0B150A}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1531,7 +2292,7 @@
       </c>
       <c r="F2" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D2)</f>
-        <v>399</v>
+        <v>588</v>
       </c>
       <c r="G2" s="2"/>
     </row>
@@ -1554,7 +2315,7 @@
       </c>
       <c r="F3" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D3)</f>
-        <v>231</v>
+        <v>420</v>
       </c>
       <c r="G3" s="2"/>
     </row>
@@ -1577,7 +2338,7 @@
       </c>
       <c r="F4" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D4)</f>
-        <v>231</v>
+        <v>420</v>
       </c>
       <c r="G4" s="2"/>
     </row>
@@ -1600,7 +2361,7 @@
       </c>
       <c r="F5" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D5)</f>
-        <v>251</v>
+        <v>440</v>
       </c>
       <c r="G5" t="s">
         <v>30</v>
@@ -1625,7 +2386,7 @@
       </c>
       <c r="F6" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D6)</f>
-        <v>231</v>
+        <v>420</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>28</v>
@@ -1653,7 +2414,7 @@
       </c>
       <c r="F7" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D7)</f>
-        <v>231</v>
+        <v>420</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" t="s">
@@ -1679,7 +2440,7 @@
       </c>
       <c r="F8" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D8)</f>
-        <v>189</v>
+        <v>378</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>18</v>
@@ -1707,7 +2468,7 @@
       </c>
       <c r="F9" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D9)</f>
-        <v>189</v>
+        <v>378</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>19</v>
@@ -1735,7 +2496,7 @@
       </c>
       <c r="F10" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D10)</f>
-        <v>189</v>
+        <v>378</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>20</v>
@@ -1763,7 +2524,7 @@
       </c>
       <c r="F11" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D11)</f>
-        <v>210</v>
+        <v>399</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>23</v>
@@ -1788,7 +2549,7 @@
       </c>
       <c r="F12" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D12)</f>
-        <v>168</v>
+        <v>357</v>
       </c>
       <c r="G12" t="s">
         <v>22</v>
@@ -1816,7 +2577,7 @@
       </c>
       <c r="F13" s="2">
         <f>_xlfn.DAYS('Release Date'!$B$1,D13)</f>
-        <v>168</v>
+        <v>357</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>21</v>

</xml_diff>